<commit_message>
Linear Campos-Villareal leaf-salt reduction at 12 mM; add Pecan LWC
</commit_message>
<xml_diff>
--- a/data/literature_data/Photosynthesis Stomatal Conductance Reduction and Dry Weight Data.xlsx
+++ b/data/literature_data/Photosynthesis Stomatal Conductance Reduction and Dry Weight Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/e5e73ff6e8b2309b/Documents/SourceCode/Photo3-Plant-Salinity-Traits/data/literature_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="6_{FF5F9A53-EC15-479F-B7D8-023BD0B5887F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D2536F8F-9D00-43AF-82B5-D8B81B56BA5C}"/>
+  <xr:revisionPtr revIDLastSave="14" documentId="6_{FF5F9A53-EC15-479F-B7D8-023BD0B5887F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2BF46EFB-2C98-45D2-A3D8-9E509FBB6C58}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="2940" yWindow="2940" windowWidth="16200" windowHeight="9307" firstSheet="8" activeTab="10" xr2:uid="{C0AAE20D-2553-4379-8EED-88D25BB078BE}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" firstSheet="5" activeTab="7" xr2:uid="{C0AAE20D-2553-4379-8EED-88D25BB078BE}"/>
   </bookViews>
   <sheets>
     <sheet name="Sanchez-Ledesma Data" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,10 @@
     <sheet name="Campos-Villareal Ion Ratios" sheetId="10" r:id="rId10"/>
     <sheet name="Sanchez-Ledesma Ion Ratios" sheetId="11" r:id="rId11"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Campos-Villareal Ion Accum'!$A$3:$L$3</definedName>
+  </definedNames>
+  <calcPr calcId="191029" calcCompleted="0"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -3195,6 +3198,444 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>Riverside</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'Campos-Villareal Ion Accum'!$B$28:$B$31</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>0.08</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2.5</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>3.5</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'Campos-Villareal Ion Accum'!$E$28:$E$31</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>298.08999999999997</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>639.08000000000004</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>987.74</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1259.77</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-0BE7-44AD-8228-46670C596615}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:v>Apache</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent2"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'Campos-Villareal Ion Accum'!$B$4:$B$7</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>0.08</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2.5</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>3.5</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'Campos-Villareal Ion Accum'!$E$4:$E$7</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>163.99</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>317.24</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>443.68</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>665.9</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-0BE7-44AD-8228-46670C596615}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:v>SVA1</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent3"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'Campos-Villareal Ion Accum'!$B$52:$B$55</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>0.08</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2.5</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>3.5</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'Campos-Villareal Ion Accum'!$E$52:$E$55</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>254.02</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>947.51</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>951.34</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>981.99</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-0BE7-44AD-8228-46670C596615}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="287927616"/>
+        <c:axId val="1803371824"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="287927616"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1803371824"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="1803371824"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="287927616"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
@@ -3276,6 +3717,46 @@
 </file>
 
 <file path=xl/charts/colors3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors4.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
   <a:schemeClr val="accent2"/>
@@ -4863,6 +5344,522 @@
 </cs:chartStyle>
 </file>
 
+<file path=xl/charts/style4.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
 <file path=xl/chartsheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <chartsheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" xr:uid="{A1FAB655-0C0B-413A-A9B0-46A99E816DBB}">
   <sheetPr/>
@@ -4891,7 +5888,7 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:absoluteAnchor>
     <xdr:pos x="0" y="0"/>
-    <xdr:ext cx="8636000" cy="6278563"/>
+    <xdr:ext cx="8654612" cy="6278836"/>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
         <xdr:cNvPr id="2" name="Chart 1">
@@ -4924,7 +5921,7 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:absoluteAnchor>
     <xdr:pos x="0" y="0"/>
-    <xdr:ext cx="8636000" cy="6278563"/>
+    <xdr:ext cx="8647206" cy="6275294"/>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
         <xdr:cNvPr id="2" name="Chart 1">
@@ -4957,7 +5954,7 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:absoluteAnchor>
     <xdr:pos x="0" y="0"/>
-    <xdr:ext cx="8636000" cy="6278563"/>
+    <xdr:ext cx="8647206" cy="6275294"/>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
         <xdr:cNvPr id="2" name="Chart 1">
@@ -5077,6 +6074,51 @@
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>135730</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>52388</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>23</xdr:col>
+      <xdr:colOff>173830</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>80963</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{533AC4CF-FD0E-818E-B1A9-23511536BCF7}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -6557,6 +7599,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD8C19C1-A04A-491D-9968-DEDC95C2A8FF}">
   <dimension ref="A1:L99"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="5" max="5" width="12.1328125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
@@ -6608,7 +7653,7 @@
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B4">
         <v>0.08</v>
@@ -6620,10 +7665,10 @@
         <v>52</v>
       </c>
       <c r="E4">
-        <v>298.08999999999997</v>
+        <v>163.99</v>
       </c>
       <c r="F4">
-        <v>97.7</v>
+        <v>90.04</v>
       </c>
       <c r="G4" t="s">
         <v>53</v>
@@ -6646,10 +7691,10 @@
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B5">
-        <v>0.08</v>
+        <v>2.5</v>
       </c>
       <c r="C5" t="s">
         <v>51</v>
@@ -6658,10 +7703,10 @@
         <v>52</v>
       </c>
       <c r="E5">
-        <v>254.02</v>
+        <v>317.24</v>
       </c>
       <c r="F5">
-        <v>95.79</v>
+        <v>90.04</v>
       </c>
       <c r="G5" t="s">
         <v>53</v>
@@ -6687,7 +7732,7 @@
         <v>7</v>
       </c>
       <c r="B6">
-        <v>0.08</v>
+        <v>3</v>
       </c>
       <c r="C6" t="s">
         <v>51</v>
@@ -6696,10 +7741,10 @@
         <v>52</v>
       </c>
       <c r="E6">
-        <v>163.99</v>
+        <v>443.68</v>
       </c>
       <c r="F6">
-        <v>90.04</v>
+        <v>91.95</v>
       </c>
       <c r="G6" t="s">
         <v>53</v>
@@ -6722,10 +7767,10 @@
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="B7">
-        <v>0.08</v>
+        <v>3.5</v>
       </c>
       <c r="C7" t="s">
         <v>51</v>
@@ -6734,10 +7779,10 @@
         <v>52</v>
       </c>
       <c r="E7">
-        <v>319.16000000000003</v>
+        <v>665.9</v>
       </c>
       <c r="F7">
-        <v>91.95</v>
+        <v>90.04</v>
       </c>
       <c r="G7" t="s">
         <v>53</v>
@@ -6760,22 +7805,22 @@
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B8">
-        <v>2.5</v>
+        <v>0.08</v>
       </c>
       <c r="C8" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="D8" t="s">
         <v>52</v>
       </c>
       <c r="E8">
-        <v>639.08000000000004</v>
+        <v>397.23</v>
       </c>
       <c r="F8">
-        <v>95.79</v>
+        <v>84.34</v>
       </c>
       <c r="G8" t="s">
         <v>53</v>
@@ -6787,7 +7832,7 @@
         <v>1</v>
       </c>
       <c r="J8" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="K8">
         <v>5</v>
@@ -6798,22 +7843,22 @@
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B9">
         <v>2.5</v>
       </c>
       <c r="C9" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="D9" t="s">
         <v>52</v>
       </c>
       <c r="E9">
-        <v>947.51</v>
+        <v>654.1</v>
       </c>
       <c r="F9">
-        <v>95.79</v>
+        <v>82.43</v>
       </c>
       <c r="G9" t="s">
         <v>53</v>
@@ -6825,7 +7870,7 @@
         <v>1</v>
       </c>
       <c r="J9" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="K9">
         <v>5</v>
@@ -6839,19 +7884,19 @@
         <v>7</v>
       </c>
       <c r="B10">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="C10" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="D10" t="s">
         <v>52</v>
       </c>
       <c r="E10">
-        <v>317.24</v>
+        <v>715.44</v>
       </c>
       <c r="F10">
-        <v>90.04</v>
+        <v>82.43</v>
       </c>
       <c r="G10" t="s">
         <v>53</v>
@@ -6863,7 +7908,7 @@
         <v>1</v>
       </c>
       <c r="J10" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="K10">
         <v>5</v>
@@ -6874,22 +7919,22 @@
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="B11">
-        <v>2.5</v>
+        <v>3.5</v>
       </c>
       <c r="C11" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="D11" t="s">
         <v>52</v>
       </c>
       <c r="E11">
-        <v>725.29</v>
+        <v>907.13</v>
       </c>
       <c r="F11">
-        <v>95.79</v>
+        <v>84.34</v>
       </c>
       <c r="G11" t="s">
         <v>53</v>
@@ -6901,7 +7946,7 @@
         <v>1</v>
       </c>
       <c r="J11" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="K11">
         <v>5</v>
@@ -6912,22 +7957,22 @@
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B12">
-        <v>3</v>
+        <v>0.08</v>
       </c>
       <c r="C12" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="D12" t="s">
         <v>52</v>
       </c>
       <c r="E12">
-        <v>987.74</v>
+        <v>338.24</v>
       </c>
       <c r="F12">
-        <v>95.79</v>
+        <v>65.900000000000006</v>
       </c>
       <c r="G12" t="s">
         <v>53</v>
@@ -6939,7 +7984,7 @@
         <v>1</v>
       </c>
       <c r="J12" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="K12">
         <v>5</v>
@@ -6950,22 +7995,22 @@
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B13">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="C13" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="D13" t="s">
         <v>52</v>
       </c>
       <c r="E13">
-        <v>951.34</v>
+        <v>455.67</v>
       </c>
       <c r="F13">
-        <v>93.87</v>
+        <v>67.099999999999994</v>
       </c>
       <c r="G13" t="s">
         <v>53</v>
@@ -6977,7 +8022,7 @@
         <v>1</v>
       </c>
       <c r="J13" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="K13">
         <v>5</v>
@@ -6994,16 +8039,16 @@
         <v>3</v>
       </c>
       <c r="C14" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="D14" t="s">
         <v>52</v>
       </c>
       <c r="E14">
-        <v>443.68</v>
+        <v>707.29</v>
       </c>
       <c r="F14">
-        <v>91.95</v>
+        <v>65.900000000000006</v>
       </c>
       <c r="G14" t="s">
         <v>53</v>
@@ -7015,7 +8060,7 @@
         <v>1</v>
       </c>
       <c r="J14" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="K14">
         <v>5</v>
@@ -7026,22 +8071,22 @@
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="B15">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="C15" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="D15" t="s">
         <v>52</v>
       </c>
       <c r="E15">
-        <v>483.91</v>
+        <v>712.08</v>
       </c>
       <c r="F15">
-        <v>95.79</v>
+        <v>67.099999999999994</v>
       </c>
       <c r="G15" t="s">
         <v>53</v>
@@ -7053,7 +8098,7 @@
         <v>1</v>
       </c>
       <c r="J15" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="K15">
         <v>5</v>
@@ -7064,22 +8109,22 @@
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B16">
-        <v>3.5</v>
+        <v>0.08</v>
       </c>
       <c r="C16" t="s">
         <v>51</v>
       </c>
       <c r="D16" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="E16">
-        <v>1259.77</v>
+        <v>12.61</v>
       </c>
       <c r="F16">
-        <v>93.87</v>
+        <v>2.78</v>
       </c>
       <c r="G16" t="s">
         <v>53</v>
@@ -7088,13 +8133,13 @@
         <v>54</v>
       </c>
       <c r="I16">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J16" t="s">
         <v>55</v>
       </c>
       <c r="K16">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L16" t="s">
         <v>56</v>
@@ -7102,22 +8147,22 @@
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B17">
-        <v>3.5</v>
+        <v>2.5</v>
       </c>
       <c r="C17" t="s">
         <v>51</v>
       </c>
       <c r="D17" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="E17">
-        <v>981.99</v>
+        <v>27.55</v>
       </c>
       <c r="F17">
-        <v>95.79</v>
+        <v>2.78</v>
       </c>
       <c r="G17" t="s">
         <v>53</v>
@@ -7126,13 +8171,13 @@
         <v>54</v>
       </c>
       <c r="I17">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J17" t="s">
         <v>55</v>
       </c>
       <c r="K17">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L17" t="s">
         <v>56</v>
@@ -7143,19 +8188,19 @@
         <v>7</v>
       </c>
       <c r="B18">
-        <v>3.5</v>
+        <v>3</v>
       </c>
       <c r="C18" t="s">
         <v>51</v>
       </c>
       <c r="D18" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="E18">
-        <v>665.9</v>
+        <v>33.1</v>
       </c>
       <c r="F18">
-        <v>90.04</v>
+        <v>2.78</v>
       </c>
       <c r="G18" t="s">
         <v>53</v>
@@ -7164,13 +8209,13 @@
         <v>54</v>
       </c>
       <c r="I18">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J18" t="s">
         <v>55</v>
       </c>
       <c r="K18">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L18" t="s">
         <v>56</v>
@@ -7178,7 +8223,7 @@
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A19" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="B19">
         <v>3.5</v>
@@ -7187,13 +8232,13 @@
         <v>51</v>
       </c>
       <c r="D19" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="E19">
-        <v>717.62</v>
+        <v>38.28</v>
       </c>
       <c r="F19">
-        <v>95.79</v>
+        <v>2.87</v>
       </c>
       <c r="G19" t="s">
         <v>53</v>
@@ -7202,13 +8247,13 @@
         <v>54</v>
       </c>
       <c r="I19">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J19" t="s">
         <v>55</v>
       </c>
       <c r="K19">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L19" t="s">
         <v>56</v>
@@ -7216,7 +8261,7 @@
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A20" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B20">
         <v>0.08</v>
@@ -7225,13 +8270,13 @@
         <v>57</v>
       </c>
       <c r="D20" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="E20">
-        <v>259.20999999999998</v>
+        <v>22.66</v>
       </c>
       <c r="F20">
-        <v>93.93</v>
+        <v>2.59</v>
       </c>
       <c r="G20" t="s">
         <v>53</v>
@@ -7240,13 +8285,13 @@
         <v>54</v>
       </c>
       <c r="I20">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J20" t="s">
         <v>58</v>
       </c>
       <c r="K20">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L20" t="s">
         <v>56</v>
@@ -7254,22 +8299,22 @@
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A21" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B21">
-        <v>0.08</v>
+        <v>2.5</v>
       </c>
       <c r="C21" t="s">
         <v>57</v>
       </c>
       <c r="D21" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="E21">
-        <v>414.48</v>
+        <v>23.67</v>
       </c>
       <c r="F21">
-        <v>84.34</v>
+        <v>2.52</v>
       </c>
       <c r="G21" t="s">
         <v>53</v>
@@ -7278,13 +8323,13 @@
         <v>54</v>
       </c>
       <c r="I21">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J21" t="s">
         <v>58</v>
       </c>
       <c r="K21">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L21" t="s">
         <v>56</v>
@@ -7295,19 +8340,19 @@
         <v>7</v>
       </c>
       <c r="B22">
-        <v>0.08</v>
+        <v>3</v>
       </c>
       <c r="C22" t="s">
         <v>57</v>
       </c>
       <c r="D22" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="E22">
-        <v>397.23</v>
+        <v>26.68</v>
       </c>
       <c r="F22">
-        <v>84.34</v>
+        <v>2.52</v>
       </c>
       <c r="G22" t="s">
         <v>53</v>
@@ -7316,13 +8361,13 @@
         <v>54</v>
       </c>
       <c r="I22">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J22" t="s">
         <v>58</v>
       </c>
       <c r="K22">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L22" t="s">
         <v>56</v>
@@ -7330,22 +8375,22 @@
     </row>
     <row r="23" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="B23">
-        <v>0.08</v>
+        <v>3.5</v>
       </c>
       <c r="C23" t="s">
         <v>57</v>
       </c>
       <c r="D23" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="E23">
-        <v>422.15</v>
+        <v>34.729999999999997</v>
       </c>
       <c r="F23">
-        <v>84.34</v>
+        <v>2.66</v>
       </c>
       <c r="G23" t="s">
         <v>53</v>
@@ -7354,13 +8399,13 @@
         <v>54</v>
       </c>
       <c r="I23">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J23" t="s">
         <v>58</v>
       </c>
       <c r="K23">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L23" t="s">
         <v>56</v>
@@ -7368,22 +8413,22 @@
     </row>
     <row r="24" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B24">
-        <v>2.5</v>
+        <v>0.08</v>
       </c>
       <c r="C24" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="D24" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="E24">
-        <v>596.59</v>
+        <v>26.32</v>
       </c>
       <c r="F24">
-        <v>93.93</v>
+        <v>2.0099999999999998</v>
       </c>
       <c r="G24" t="s">
         <v>53</v>
@@ -7392,13 +8437,13 @@
         <v>54</v>
       </c>
       <c r="I24">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J24" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="K24">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L24" t="s">
         <v>56</v>
@@ -7406,22 +8451,22 @@
     </row>
     <row r="25" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B25">
         <v>2.5</v>
       </c>
       <c r="C25" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="D25" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="E25">
-        <v>709.69</v>
+        <v>29.06</v>
       </c>
       <c r="F25">
-        <v>86.26</v>
+        <v>2.0099999999999998</v>
       </c>
       <c r="G25" t="s">
         <v>53</v>
@@ -7430,13 +8475,13 @@
         <v>54</v>
       </c>
       <c r="I25">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J25" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="K25">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L25" t="s">
         <v>56</v>
@@ -7447,19 +8492,19 @@
         <v>7</v>
       </c>
       <c r="B26">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="C26" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="D26" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="E26">
-        <v>654.1</v>
+        <v>32.36</v>
       </c>
       <c r="F26">
-        <v>82.43</v>
+        <v>2.08</v>
       </c>
       <c r="G26" t="s">
         <v>53</v>
@@ -7468,13 +8513,13 @@
         <v>54</v>
       </c>
       <c r="I26">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J26" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="K26">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L26" t="s">
         <v>56</v>
@@ -7482,22 +8527,22 @@
     </row>
     <row r="27" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A27" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="B27">
-        <v>2.5</v>
+        <v>3.5</v>
       </c>
       <c r="C27" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="D27" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="E27">
-        <v>748.03</v>
+        <v>46.59</v>
       </c>
       <c r="F27">
-        <v>86.26</v>
+        <v>2.08</v>
       </c>
       <c r="G27" t="s">
         <v>53</v>
@@ -7506,13 +8551,13 @@
         <v>54</v>
       </c>
       <c r="I27">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J27" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="K27">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L27" t="s">
         <v>56</v>
@@ -7523,19 +8568,19 @@
         <v>8</v>
       </c>
       <c r="B28">
-        <v>3</v>
+        <v>0.08</v>
       </c>
       <c r="C28" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="D28" t="s">
         <v>52</v>
       </c>
       <c r="E28">
-        <v>987.65</v>
+        <v>298.08999999999997</v>
       </c>
       <c r="F28">
-        <v>90.1</v>
+        <v>97.7</v>
       </c>
       <c r="G28" t="s">
         <v>53</v>
@@ -7547,7 +8592,7 @@
         <v>1</v>
       </c>
       <c r="J28" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="K28">
         <v>5</v>
@@ -7558,22 +8603,22 @@
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A29" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B29">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="C29" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="D29" t="s">
         <v>52</v>
       </c>
       <c r="E29">
-        <v>878.38</v>
+        <v>639.08000000000004</v>
       </c>
       <c r="F29">
-        <v>86.26</v>
+        <v>95.79</v>
       </c>
       <c r="G29" t="s">
         <v>53</v>
@@ -7585,7 +8630,7 @@
         <v>1</v>
       </c>
       <c r="J29" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="K29">
         <v>5</v>
@@ -7596,22 +8641,22 @@
     </row>
     <row r="30" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A30" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B30">
         <v>3</v>
       </c>
       <c r="C30" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="D30" t="s">
         <v>52</v>
       </c>
       <c r="E30">
-        <v>715.44</v>
+        <v>987.74</v>
       </c>
       <c r="F30">
-        <v>82.43</v>
+        <v>95.79</v>
       </c>
       <c r="G30" t="s">
         <v>53</v>
@@ -7623,7 +8668,7 @@
         <v>1</v>
       </c>
       <c r="J30" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="K30">
         <v>5</v>
@@ -7634,22 +8679,22 @@
     </row>
     <row r="31" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A31" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B31">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="C31" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="D31" t="s">
         <v>52</v>
       </c>
       <c r="E31">
-        <v>713.53</v>
+        <v>1259.77</v>
       </c>
       <c r="F31">
-        <v>84.34</v>
+        <v>93.87</v>
       </c>
       <c r="G31" t="s">
         <v>53</v>
@@ -7661,7 +8706,7 @@
         <v>1</v>
       </c>
       <c r="J31" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="K31">
         <v>5</v>
@@ -7675,7 +8720,7 @@
         <v>8</v>
       </c>
       <c r="B32">
-        <v>3.5</v>
+        <v>0.08</v>
       </c>
       <c r="C32" t="s">
         <v>57</v>
@@ -7684,10 +8729,10 @@
         <v>52</v>
       </c>
       <c r="E32">
-        <v>1359.53</v>
+        <v>259.20999999999998</v>
       </c>
       <c r="F32">
-        <v>92.01</v>
+        <v>93.93</v>
       </c>
       <c r="G32" t="s">
         <v>53</v>
@@ -7710,10 +8755,10 @@
     </row>
     <row r="33" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A33" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B33">
-        <v>3.5</v>
+        <v>2.5</v>
       </c>
       <c r="C33" t="s">
         <v>57</v>
@@ -7722,10 +8767,10 @@
         <v>52</v>
       </c>
       <c r="E33">
-        <v>882.21</v>
+        <v>596.59</v>
       </c>
       <c r="F33">
-        <v>84.34</v>
+        <v>93.93</v>
       </c>
       <c r="G33" t="s">
         <v>53</v>
@@ -7748,10 +8793,10 @@
     </row>
     <row r="34" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A34" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B34">
-        <v>3.5</v>
+        <v>3</v>
       </c>
       <c r="C34" t="s">
         <v>57</v>
@@ -7760,10 +8805,10 @@
         <v>52</v>
       </c>
       <c r="E34">
-        <v>907.13</v>
+        <v>987.65</v>
       </c>
       <c r="F34">
-        <v>84.34</v>
+        <v>90.1</v>
       </c>
       <c r="G34" t="s">
         <v>53</v>
@@ -7786,7 +8831,7 @@
     </row>
     <row r="35" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A35" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B35">
         <v>3.5</v>
@@ -7798,10 +8843,10 @@
         <v>52</v>
       </c>
       <c r="E35">
-        <v>836.21</v>
+        <v>1359.53</v>
       </c>
       <c r="F35">
-        <v>82.43</v>
+        <v>92.01</v>
       </c>
       <c r="G35" t="s">
         <v>53</v>
@@ -7862,10 +8907,10 @@
     </row>
     <row r="37" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A37" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B37">
-        <v>0.08</v>
+        <v>2.5</v>
       </c>
       <c r="C37" t="s">
         <v>59</v>
@@ -7874,10 +8919,10 @@
         <v>52</v>
       </c>
       <c r="E37">
-        <v>377.78</v>
+        <v>652.16999999999996</v>
       </c>
       <c r="F37">
-        <v>64.7</v>
+        <v>70.69</v>
       </c>
       <c r="G37" t="s">
         <v>53</v>
@@ -7900,10 +8945,10 @@
     </row>
     <row r="38" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A38" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B38">
-        <v>0.08</v>
+        <v>3</v>
       </c>
       <c r="C38" t="s">
         <v>59</v>
@@ -7912,10 +8957,10 @@
         <v>52</v>
       </c>
       <c r="E38">
-        <v>338.24</v>
+        <v>839.1</v>
       </c>
       <c r="F38">
-        <v>65.900000000000006</v>
+        <v>71.89</v>
       </c>
       <c r="G38" t="s">
         <v>53</v>
@@ -7938,10 +8983,10 @@
     </row>
     <row r="39" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A39" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B39">
-        <v>0.08</v>
+        <v>3.5</v>
       </c>
       <c r="C39" t="s">
         <v>59</v>
@@ -7950,10 +8995,10 @@
         <v>52</v>
       </c>
       <c r="E39">
-        <v>454.47</v>
+        <v>815.13</v>
       </c>
       <c r="F39">
-        <v>68.3</v>
+        <v>70.69</v>
       </c>
       <c r="G39" t="s">
         <v>53</v>
@@ -7979,19 +9024,19 @@
         <v>8</v>
       </c>
       <c r="B40">
-        <v>2.5</v>
+        <v>0.08</v>
       </c>
       <c r="C40" t="s">
-        <v>59</v>
+        <v>51</v>
       </c>
       <c r="D40" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="E40">
-        <v>652.16999999999996</v>
+        <v>22.57</v>
       </c>
       <c r="F40">
-        <v>70.69</v>
+        <v>3.35</v>
       </c>
       <c r="G40" t="s">
         <v>53</v>
@@ -8000,13 +9045,13 @@
         <v>54</v>
       </c>
       <c r="I40">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J40" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="K40">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L40" t="s">
         <v>56</v>
@@ -8014,22 +9059,22 @@
     </row>
     <row r="41" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A41" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B41">
         <v>2.5</v>
       </c>
       <c r="C41" t="s">
-        <v>59</v>
+        <v>51</v>
       </c>
       <c r="D41" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="E41">
-        <v>595.86</v>
+        <v>34.06</v>
       </c>
       <c r="F41">
-        <v>67.099999999999994</v>
+        <v>3.35</v>
       </c>
       <c r="G41" t="s">
         <v>53</v>
@@ -8038,13 +9083,13 @@
         <v>54</v>
       </c>
       <c r="I41">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J41" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="K41">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L41" t="s">
         <v>56</v>
@@ -8052,22 +9097,22 @@
     </row>
     <row r="42" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A42" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B42">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="C42" t="s">
-        <v>59</v>
+        <v>51</v>
       </c>
       <c r="D42" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="E42">
-        <v>455.67</v>
+        <v>51.69</v>
       </c>
       <c r="F42">
-        <v>67.099999999999994</v>
+        <v>3.54</v>
       </c>
       <c r="G42" t="s">
         <v>53</v>
@@ -8076,13 +9121,13 @@
         <v>54</v>
       </c>
       <c r="I42">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J42" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="K42">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L42" t="s">
         <v>56</v>
@@ -8090,22 +9135,22 @@
     </row>
     <row r="43" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A43" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B43">
-        <v>2.5</v>
+        <v>3.5</v>
       </c>
       <c r="C43" t="s">
-        <v>59</v>
+        <v>51</v>
       </c>
       <c r="D43" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="E43">
-        <v>837.9</v>
+        <v>58.97</v>
       </c>
       <c r="F43">
-        <v>65.900000000000006</v>
+        <v>3.35</v>
       </c>
       <c r="G43" t="s">
         <v>53</v>
@@ -8114,13 +9159,13 @@
         <v>54</v>
       </c>
       <c r="I43">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J43" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="K43">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L43" t="s">
         <v>56</v>
@@ -8131,19 +9176,19 @@
         <v>8</v>
       </c>
       <c r="B44">
-        <v>3</v>
+        <v>0.08</v>
       </c>
       <c r="C44" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="D44" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="E44">
-        <v>839.1</v>
+        <v>21.8</v>
       </c>
       <c r="F44">
-        <v>71.89</v>
+        <v>3.09</v>
       </c>
       <c r="G44" t="s">
         <v>53</v>
@@ -8152,13 +9197,13 @@
         <v>54</v>
       </c>
       <c r="I44">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J44" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="K44">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L44" t="s">
         <v>56</v>
@@ -8166,22 +9211,22 @@
     </row>
     <row r="45" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A45" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B45">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="C45" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="D45" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="E45">
-        <v>677.34</v>
+        <v>27.26</v>
       </c>
       <c r="F45">
-        <v>64.7</v>
+        <v>3.09</v>
       </c>
       <c r="G45" t="s">
         <v>53</v>
@@ -8190,13 +9235,13 @@
         <v>54</v>
       </c>
       <c r="I45">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J45" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="K45">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L45" t="s">
         <v>56</v>
@@ -8204,22 +9249,22 @@
     </row>
     <row r="46" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A46" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B46">
         <v>3</v>
       </c>
       <c r="C46" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="D46" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="E46">
-        <v>707.29</v>
+        <v>38.61</v>
       </c>
       <c r="F46">
-        <v>65.900000000000006</v>
+        <v>2.95</v>
       </c>
       <c r="G46" t="s">
         <v>53</v>
@@ -8228,13 +9273,13 @@
         <v>54</v>
       </c>
       <c r="I46">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J46" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="K46">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L46" t="s">
         <v>56</v>
@@ -8242,22 +9287,22 @@
     </row>
     <row r="47" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A47" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B47">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="C47" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="D47" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="E47">
-        <v>837.9</v>
+        <v>41.2</v>
       </c>
       <c r="F47">
-        <v>68.3</v>
+        <v>2.87</v>
       </c>
       <c r="G47" t="s">
         <v>53</v>
@@ -8266,13 +9311,13 @@
         <v>54</v>
       </c>
       <c r="I47">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J47" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="K47">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L47" t="s">
         <v>56</v>
@@ -8283,19 +9328,19 @@
         <v>8</v>
       </c>
       <c r="B48">
-        <v>3.5</v>
+        <v>0.08</v>
       </c>
       <c r="C48" t="s">
         <v>59</v>
       </c>
       <c r="D48" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="E48">
-        <v>815.13</v>
+        <v>27.47</v>
       </c>
       <c r="F48">
-        <v>70.69</v>
+        <v>2.23</v>
       </c>
       <c r="G48" t="s">
         <v>53</v>
@@ -8304,13 +9349,13 @@
         <v>54</v>
       </c>
       <c r="I48">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J48" t="s">
         <v>60</v>
       </c>
       <c r="K48">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L48" t="s">
         <v>56</v>
@@ -8318,22 +9363,22 @@
     </row>
     <row r="49" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A49" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B49">
-        <v>3.5</v>
+        <v>2.5</v>
       </c>
       <c r="C49" t="s">
         <v>59</v>
       </c>
       <c r="D49" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="E49">
-        <v>619.82000000000005</v>
+        <v>25.89</v>
       </c>
       <c r="F49">
-        <v>64.7</v>
+        <v>2.37</v>
       </c>
       <c r="G49" t="s">
         <v>53</v>
@@ -8342,13 +9387,13 @@
         <v>54</v>
       </c>
       <c r="I49">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J49" t="s">
         <v>60</v>
       </c>
       <c r="K49">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L49" t="s">
         <v>56</v>
@@ -8356,22 +9401,22 @@
     </row>
     <row r="50" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A50" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B50">
-        <v>3.5</v>
+        <v>3</v>
       </c>
       <c r="C50" t="s">
         <v>59</v>
       </c>
       <c r="D50" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="E50">
-        <v>712.08</v>
+        <v>31.93</v>
       </c>
       <c r="F50">
-        <v>67.099999999999994</v>
+        <v>2.23</v>
       </c>
       <c r="G50" t="s">
         <v>53</v>
@@ -8380,13 +9425,13 @@
         <v>54</v>
       </c>
       <c r="I50">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J50" t="s">
         <v>60</v>
       </c>
       <c r="K50">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L50" t="s">
         <v>56</v>
@@ -8394,7 +9439,7 @@
     </row>
     <row r="51" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A51" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B51">
         <v>3.5</v>
@@ -8403,13 +9448,13 @@
         <v>59</v>
       </c>
       <c r="D51" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="E51">
-        <v>809.14</v>
+        <v>31.21</v>
       </c>
       <c r="F51">
-        <v>64.7</v>
+        <v>2.37</v>
       </c>
       <c r="G51" t="s">
         <v>53</v>
@@ -8418,13 +9463,13 @@
         <v>54</v>
       </c>
       <c r="I51">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J51" t="s">
         <v>60</v>
       </c>
       <c r="K51">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L51" t="s">
         <v>56</v>
@@ -8432,7 +9477,7 @@
     </row>
     <row r="52" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A52" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B52">
         <v>0.08</v>
@@ -8441,13 +9486,13 @@
         <v>51</v>
       </c>
       <c r="D52" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
       <c r="E52">
-        <v>22.57</v>
+        <v>254.02</v>
       </c>
       <c r="F52">
-        <v>3.35</v>
+        <v>95.79</v>
       </c>
       <c r="G52" t="s">
         <v>53</v>
@@ -8456,13 +9501,13 @@
         <v>54</v>
       </c>
       <c r="I52">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J52" t="s">
         <v>55</v>
       </c>
       <c r="K52">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L52" t="s">
         <v>56</v>
@@ -8473,19 +9518,19 @@
         <v>9</v>
       </c>
       <c r="B53">
-        <v>0.08</v>
+        <v>2.5</v>
       </c>
       <c r="C53" t="s">
         <v>51</v>
       </c>
       <c r="D53" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
       <c r="E53">
-        <v>16.72</v>
+        <v>947.51</v>
       </c>
       <c r="F53">
-        <v>2.87</v>
+        <v>95.79</v>
       </c>
       <c r="G53" t="s">
         <v>53</v>
@@ -8494,13 +9539,13 @@
         <v>54</v>
       </c>
       <c r="I53">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J53" t="s">
         <v>55</v>
       </c>
       <c r="K53">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L53" t="s">
         <v>56</v>
@@ -8508,22 +9553,22 @@
     </row>
     <row r="54" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A54" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B54">
-        <v>0.08</v>
+        <v>3</v>
       </c>
       <c r="C54" t="s">
         <v>51</v>
       </c>
       <c r="D54" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
       <c r="E54">
-        <v>12.61</v>
+        <v>951.34</v>
       </c>
       <c r="F54">
-        <v>2.78</v>
+        <v>93.87</v>
       </c>
       <c r="G54" t="s">
         <v>53</v>
@@ -8532,13 +9577,13 @@
         <v>54</v>
       </c>
       <c r="I54">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J54" t="s">
         <v>55</v>
       </c>
       <c r="K54">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L54" t="s">
         <v>56</v>
@@ -8546,22 +9591,22 @@
     </row>
     <row r="55" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A55" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B55">
-        <v>0.08</v>
+        <v>3.5</v>
       </c>
       <c r="C55" t="s">
         <v>51</v>
       </c>
       <c r="D55" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
       <c r="E55">
-        <v>15.96</v>
+        <v>981.99</v>
       </c>
       <c r="F55">
-        <v>2.87</v>
+        <v>95.79</v>
       </c>
       <c r="G55" t="s">
         <v>53</v>
@@ -8570,13 +9615,13 @@
         <v>54</v>
       </c>
       <c r="I55">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J55" t="s">
         <v>55</v>
       </c>
       <c r="K55">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L55" t="s">
         <v>56</v>
@@ -8584,22 +9629,22 @@
     </row>
     <row r="56" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A56" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B56">
-        <v>2.5</v>
+        <v>0.08</v>
       </c>
       <c r="C56" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="D56" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
       <c r="E56">
-        <v>34.06</v>
+        <v>414.48</v>
       </c>
       <c r="F56">
-        <v>3.35</v>
+        <v>84.34</v>
       </c>
       <c r="G56" t="s">
         <v>53</v>
@@ -8608,13 +9653,13 @@
         <v>54</v>
       </c>
       <c r="I56">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J56" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="K56">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L56" t="s">
         <v>56</v>
@@ -8628,16 +9673,16 @@
         <v>2.5</v>
       </c>
       <c r="C57" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="D57" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
       <c r="E57">
-        <v>37.03</v>
+        <v>709.69</v>
       </c>
       <c r="F57">
-        <v>2.87</v>
+        <v>86.26</v>
       </c>
       <c r="G57" t="s">
         <v>53</v>
@@ -8646,13 +9691,13 @@
         <v>54</v>
       </c>
       <c r="I57">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J57" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="K57">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L57" t="s">
         <v>56</v>
@@ -8660,22 +9705,22 @@
     </row>
     <row r="58" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A58" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B58">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="C58" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="D58" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
       <c r="E58">
-        <v>27.55</v>
+        <v>878.38</v>
       </c>
       <c r="F58">
-        <v>2.78</v>
+        <v>86.26</v>
       </c>
       <c r="G58" t="s">
         <v>53</v>
@@ -8684,13 +9729,13 @@
         <v>54</v>
       </c>
       <c r="I58">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J58" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="K58">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L58" t="s">
         <v>56</v>
@@ -8698,22 +9743,22 @@
     </row>
     <row r="59" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A59" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B59">
-        <v>2.5</v>
+        <v>3.5</v>
       </c>
       <c r="C59" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="D59" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
       <c r="E59">
-        <v>34.729999999999997</v>
+        <v>882.21</v>
       </c>
       <c r="F59">
-        <v>2.87</v>
+        <v>84.34</v>
       </c>
       <c r="G59" t="s">
         <v>53</v>
@@ -8722,13 +9767,13 @@
         <v>54</v>
       </c>
       <c r="I59">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J59" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="K59">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L59" t="s">
         <v>56</v>
@@ -8736,22 +9781,22 @@
     </row>
     <row r="60" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A60" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B60">
-        <v>3</v>
+        <v>0.08</v>
       </c>
       <c r="C60" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="D60" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
       <c r="E60">
-        <v>51.69</v>
+        <v>377.78</v>
       </c>
       <c r="F60">
-        <v>3.54</v>
+        <v>64.7</v>
       </c>
       <c r="G60" t="s">
         <v>53</v>
@@ -8760,13 +9805,13 @@
         <v>54</v>
       </c>
       <c r="I60">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J60" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="K60">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L60" t="s">
         <v>56</v>
@@ -8777,19 +9822,19 @@
         <v>9</v>
       </c>
       <c r="B61">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="C61" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="D61" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
       <c r="E61">
-        <v>62.13</v>
+        <v>595.86</v>
       </c>
       <c r="F61">
-        <v>2.87</v>
+        <v>67.099999999999994</v>
       </c>
       <c r="G61" t="s">
         <v>53</v>
@@ -8798,13 +9843,13 @@
         <v>54</v>
       </c>
       <c r="I61">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J61" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="K61">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L61" t="s">
         <v>56</v>
@@ -8812,22 +9857,22 @@
     </row>
     <row r="62" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A62" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B62">
         <v>3</v>
       </c>
       <c r="C62" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="D62" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
       <c r="E62">
-        <v>33.1</v>
+        <v>677.34</v>
       </c>
       <c r="F62">
-        <v>2.78</v>
+        <v>64.7</v>
       </c>
       <c r="G62" t="s">
         <v>53</v>
@@ -8836,13 +9881,13 @@
         <v>54</v>
       </c>
       <c r="I62">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J62" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="K62">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L62" t="s">
         <v>56</v>
@@ -8850,22 +9895,22 @@
     </row>
     <row r="63" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A63" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B63">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="C63" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="D63" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
       <c r="E63">
-        <v>37.799999999999997</v>
+        <v>619.82000000000005</v>
       </c>
       <c r="F63">
-        <v>2.87</v>
+        <v>64.7</v>
       </c>
       <c r="G63" t="s">
         <v>53</v>
@@ -8874,13 +9919,13 @@
         <v>54</v>
       </c>
       <c r="I63">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J63" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="K63">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L63" t="s">
         <v>56</v>
@@ -8888,10 +9933,10 @@
     </row>
     <row r="64" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A64" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B64">
-        <v>3.5</v>
+        <v>0.08</v>
       </c>
       <c r="C64" t="s">
         <v>51</v>
@@ -8900,10 +9945,10 @@
         <v>61</v>
       </c>
       <c r="E64">
-        <v>58.97</v>
+        <v>16.72</v>
       </c>
       <c r="F64">
-        <v>3.35</v>
+        <v>2.87</v>
       </c>
       <c r="G64" t="s">
         <v>53</v>
@@ -8929,7 +9974,7 @@
         <v>9</v>
       </c>
       <c r="B65">
-        <v>3.5</v>
+        <v>2.5</v>
       </c>
       <c r="C65" t="s">
         <v>51</v>
@@ -8938,7 +9983,7 @@
         <v>61</v>
       </c>
       <c r="E65">
-        <v>67.87</v>
+        <v>37.03</v>
       </c>
       <c r="F65">
         <v>2.87</v>
@@ -8964,10 +10009,10 @@
     </row>
     <row r="66" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A66" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B66">
-        <v>3.5</v>
+        <v>3</v>
       </c>
       <c r="C66" t="s">
         <v>51</v>
@@ -8976,7 +10021,7 @@
         <v>61</v>
       </c>
       <c r="E66">
-        <v>38.28</v>
+        <v>62.13</v>
       </c>
       <c r="F66">
         <v>2.87</v>
@@ -9002,7 +10047,7 @@
     </row>
     <row r="67" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A67" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B67">
         <v>3.5</v>
@@ -9014,10 +10059,10 @@
         <v>61</v>
       </c>
       <c r="E67">
-        <v>38.75</v>
+        <v>67.87</v>
       </c>
       <c r="F67">
-        <v>2.97</v>
+        <v>2.87</v>
       </c>
       <c r="G67" t="s">
         <v>53</v>
@@ -9040,7 +10085,7 @@
     </row>
     <row r="68" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A68" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B68">
         <v>0.08</v>
@@ -9052,10 +10097,10 @@
         <v>61</v>
       </c>
       <c r="E68">
-        <v>21.8</v>
+        <v>14.39</v>
       </c>
       <c r="F68">
-        <v>3.09</v>
+        <v>2.73</v>
       </c>
       <c r="G68" t="s">
         <v>53</v>
@@ -9081,7 +10126,7 @@
         <v>9</v>
       </c>
       <c r="B69">
-        <v>0.08</v>
+        <v>2.5</v>
       </c>
       <c r="C69" t="s">
         <v>57</v>
@@ -9090,10 +10135,10 @@
         <v>61</v>
       </c>
       <c r="E69">
-        <v>14.39</v>
+        <v>29.2</v>
       </c>
       <c r="F69">
-        <v>2.73</v>
+        <v>2.59</v>
       </c>
       <c r="G69" t="s">
         <v>53</v>
@@ -9116,10 +10161,10 @@
     </row>
     <row r="70" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A70" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B70">
-        <v>0.08</v>
+        <v>3</v>
       </c>
       <c r="C70" t="s">
         <v>57</v>
@@ -9128,10 +10173,10 @@
         <v>61</v>
       </c>
       <c r="E70">
-        <v>22.66</v>
+        <v>36.24</v>
       </c>
       <c r="F70">
-        <v>2.59</v>
+        <v>2.66</v>
       </c>
       <c r="G70" t="s">
         <v>53</v>
@@ -9154,10 +10199,10 @@
     </row>
     <row r="71" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A71" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B71">
-        <v>0.08</v>
+        <v>3.5</v>
       </c>
       <c r="C71" t="s">
         <v>57</v>
@@ -9166,10 +10211,10 @@
         <v>61</v>
       </c>
       <c r="E71">
-        <v>16.12</v>
+        <v>48.17</v>
       </c>
       <c r="F71">
-        <v>2.59</v>
+        <v>2.52</v>
       </c>
       <c r="G71" t="s">
         <v>53</v>
@@ -9192,22 +10237,22 @@
     </row>
     <row r="72" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A72" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B72">
-        <v>2.5</v>
+        <v>0.08</v>
       </c>
       <c r="C72" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="D72" t="s">
         <v>61</v>
       </c>
       <c r="E72">
-        <v>27.26</v>
+        <v>40.770000000000003</v>
       </c>
       <c r="F72">
-        <v>3.09</v>
+        <v>2.0099999999999998</v>
       </c>
       <c r="G72" t="s">
         <v>53</v>
@@ -9219,7 +10264,7 @@
         <v>2</v>
       </c>
       <c r="J72" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="K72">
         <v>6</v>
@@ -9236,16 +10281,16 @@
         <v>2.5</v>
       </c>
       <c r="C73" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="D73" t="s">
         <v>61</v>
       </c>
       <c r="E73">
-        <v>29.2</v>
+        <v>50.4</v>
       </c>
       <c r="F73">
-        <v>2.59</v>
+        <v>1.94</v>
       </c>
       <c r="G73" t="s">
         <v>53</v>
@@ -9257,7 +10302,7 @@
         <v>2</v>
       </c>
       <c r="J73" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="K73">
         <v>6</v>
@@ -9268,22 +10313,22 @@
     </row>
     <row r="74" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A74" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="B74">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="C74" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="D74" t="s">
         <v>61</v>
       </c>
       <c r="E74">
-        <v>23.67</v>
+        <v>49.39</v>
       </c>
       <c r="F74">
-        <v>2.52</v>
+        <v>1.87</v>
       </c>
       <c r="G74" t="s">
         <v>53</v>
@@ -9295,7 +10340,7 @@
         <v>2</v>
       </c>
       <c r="J74" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="K74">
         <v>6</v>
@@ -9306,22 +10351,22 @@
     </row>
     <row r="75" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A75" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B75">
-        <v>2.5</v>
+        <v>3.5</v>
       </c>
       <c r="C75" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="D75" t="s">
         <v>61</v>
       </c>
       <c r="E75">
-        <v>20.14</v>
+        <v>52.41</v>
       </c>
       <c r="F75">
-        <v>2.66</v>
+        <v>1.87</v>
       </c>
       <c r="G75" t="s">
         <v>53</v>
@@ -9333,7 +10378,7 @@
         <v>2</v>
       </c>
       <c r="J75" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="K75">
         <v>6</v>
@@ -9344,22 +10389,22 @@
     </row>
     <row r="76" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A76" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B76">
-        <v>3</v>
+        <v>0.08</v>
       </c>
       <c r="C76" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="D76" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
       <c r="E76">
-        <v>38.61</v>
+        <v>319.16000000000003</v>
       </c>
       <c r="F76">
-        <v>2.95</v>
+        <v>91.95</v>
       </c>
       <c r="G76" t="s">
         <v>53</v>
@@ -9368,13 +10413,13 @@
         <v>54</v>
       </c>
       <c r="I76">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J76" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="K76">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L76" t="s">
         <v>56</v>
@@ -9382,22 +10427,22 @@
     </row>
     <row r="77" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A77" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B77">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="C77" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="D77" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
       <c r="E77">
-        <v>36.24</v>
+        <v>725.29</v>
       </c>
       <c r="F77">
-        <v>2.66</v>
+        <v>95.79</v>
       </c>
       <c r="G77" t="s">
         <v>53</v>
@@ -9406,13 +10451,13 @@
         <v>54</v>
       </c>
       <c r="I77">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J77" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="K77">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L77" t="s">
         <v>56</v>
@@ -9420,22 +10465,22 @@
     </row>
     <row r="78" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A78" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="B78">
         <v>3</v>
       </c>
       <c r="C78" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="D78" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
       <c r="E78">
-        <v>26.68</v>
+        <v>483.91</v>
       </c>
       <c r="F78">
-        <v>2.52</v>
+        <v>95.79</v>
       </c>
       <c r="G78" t="s">
         <v>53</v>
@@ -9444,13 +10489,13 @@
         <v>54</v>
       </c>
       <c r="I78">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J78" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="K78">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L78" t="s">
         <v>56</v>
@@ -9461,19 +10506,19 @@
         <v>10</v>
       </c>
       <c r="B79">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="C79" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="D79" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
       <c r="E79">
-        <v>25.89</v>
+        <v>717.62</v>
       </c>
       <c r="F79">
-        <v>2.66</v>
+        <v>95.79</v>
       </c>
       <c r="G79" t="s">
         <v>53</v>
@@ -9482,13 +10527,13 @@
         <v>54</v>
       </c>
       <c r="I79">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J79" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="K79">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L79" t="s">
         <v>56</v>
@@ -9496,22 +10541,22 @@
     </row>
     <row r="80" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A80" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B80">
-        <v>3.5</v>
+        <v>0.08</v>
       </c>
       <c r="C80" t="s">
         <v>57</v>
       </c>
       <c r="D80" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
       <c r="E80">
-        <v>41.2</v>
+        <v>422.15</v>
       </c>
       <c r="F80">
-        <v>2.87</v>
+        <v>84.34</v>
       </c>
       <c r="G80" t="s">
         <v>53</v>
@@ -9520,13 +10565,13 @@
         <v>54</v>
       </c>
       <c r="I80">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J80" t="s">
         <v>58</v>
       </c>
       <c r="K80">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L80" t="s">
         <v>56</v>
@@ -9534,22 +10579,22 @@
     </row>
     <row r="81" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A81" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B81">
-        <v>3.5</v>
+        <v>2.5</v>
       </c>
       <c r="C81" t="s">
         <v>57</v>
       </c>
       <c r="D81" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
       <c r="E81">
-        <v>48.17</v>
+        <v>748.03</v>
       </c>
       <c r="F81">
-        <v>2.52</v>
+        <v>86.26</v>
       </c>
       <c r="G81" t="s">
         <v>53</v>
@@ -9558,13 +10603,13 @@
         <v>54</v>
       </c>
       <c r="I81">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J81" t="s">
         <v>58</v>
       </c>
       <c r="K81">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L81" t="s">
         <v>56</v>
@@ -9572,22 +10617,22 @@
     </row>
     <row r="82" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A82" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="B82">
-        <v>3.5</v>
+        <v>3</v>
       </c>
       <c r="C82" t="s">
         <v>57</v>
       </c>
       <c r="D82" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
       <c r="E82">
-        <v>34.729999999999997</v>
+        <v>713.53</v>
       </c>
       <c r="F82">
-        <v>2.66</v>
+        <v>84.34</v>
       </c>
       <c r="G82" t="s">
         <v>53</v>
@@ -9596,13 +10641,13 @@
         <v>54</v>
       </c>
       <c r="I82">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J82" t="s">
         <v>58</v>
       </c>
       <c r="K82">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L82" t="s">
         <v>56</v>
@@ -9619,13 +10664,13 @@
         <v>57</v>
       </c>
       <c r="D83" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
       <c r="E83">
-        <v>27.76</v>
+        <v>836.21</v>
       </c>
       <c r="F83">
-        <v>2.59</v>
+        <v>82.43</v>
       </c>
       <c r="G83" t="s">
         <v>53</v>
@@ -9634,13 +10679,13 @@
         <v>54</v>
       </c>
       <c r="I83">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J83" t="s">
         <v>58</v>
       </c>
       <c r="K83">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L83" t="s">
         <v>56</v>
@@ -9648,7 +10693,7 @@
     </row>
     <row r="84" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A84" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B84">
         <v>0.08</v>
@@ -9657,13 +10702,13 @@
         <v>59</v>
       </c>
       <c r="D84" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
       <c r="E84">
-        <v>27.47</v>
+        <v>454.47</v>
       </c>
       <c r="F84">
-        <v>2.23</v>
+        <v>68.3</v>
       </c>
       <c r="G84" t="s">
         <v>53</v>
@@ -9672,13 +10717,13 @@
         <v>54</v>
       </c>
       <c r="I84">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J84" t="s">
         <v>60</v>
       </c>
       <c r="K84">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L84" t="s">
         <v>56</v>
@@ -9686,22 +10731,22 @@
     </row>
     <row r="85" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A85" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B85">
-        <v>0.08</v>
+        <v>2.5</v>
       </c>
       <c r="C85" t="s">
         <v>59</v>
       </c>
       <c r="D85" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
       <c r="E85">
-        <v>40.770000000000003</v>
+        <v>837.9</v>
       </c>
       <c r="F85">
-        <v>2.0099999999999998</v>
+        <v>65.900000000000006</v>
       </c>
       <c r="G85" t="s">
         <v>53</v>
@@ -9710,13 +10755,13 @@
         <v>54</v>
       </c>
       <c r="I85">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J85" t="s">
         <v>60</v>
       </c>
       <c r="K85">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L85" t="s">
         <v>56</v>
@@ -9724,22 +10769,22 @@
     </row>
     <row r="86" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A86" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="B86">
-        <v>0.08</v>
+        <v>3</v>
       </c>
       <c r="C86" t="s">
         <v>59</v>
       </c>
       <c r="D86" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
       <c r="E86">
-        <v>26.32</v>
+        <v>837.9</v>
       </c>
       <c r="F86">
-        <v>2.0099999999999998</v>
+        <v>68.3</v>
       </c>
       <c r="G86" t="s">
         <v>53</v>
@@ -9748,13 +10793,13 @@
         <v>54</v>
       </c>
       <c r="I86">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J86" t="s">
         <v>60</v>
       </c>
       <c r="K86">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L86" t="s">
         <v>56</v>
@@ -9765,19 +10810,19 @@
         <v>10</v>
       </c>
       <c r="B87">
-        <v>0.08</v>
+        <v>3.5</v>
       </c>
       <c r="C87" t="s">
         <v>59</v>
       </c>
       <c r="D87" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
       <c r="E87">
-        <v>14.03</v>
+        <v>809.14</v>
       </c>
       <c r="F87">
-        <v>2.0099999999999998</v>
+        <v>64.7</v>
       </c>
       <c r="G87" t="s">
         <v>53</v>
@@ -9786,13 +10831,13 @@
         <v>54</v>
       </c>
       <c r="I87">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J87" t="s">
         <v>60</v>
       </c>
       <c r="K87">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="L87" t="s">
         <v>56</v>
@@ -9800,22 +10845,22 @@
     </row>
     <row r="88" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A88" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B88">
-        <v>2.5</v>
+        <v>0.08</v>
       </c>
       <c r="C88" t="s">
-        <v>59</v>
+        <v>51</v>
       </c>
       <c r="D88" t="s">
         <v>61</v>
       </c>
       <c r="E88">
-        <v>25.89</v>
+        <v>15.96</v>
       </c>
       <c r="F88">
-        <v>2.37</v>
+        <v>2.87</v>
       </c>
       <c r="G88" t="s">
         <v>53</v>
@@ -9827,7 +10872,7 @@
         <v>2</v>
       </c>
       <c r="J88" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="K88">
         <v>6</v>
@@ -9838,22 +10883,22 @@
     </row>
     <row r="89" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A89" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B89">
         <v>2.5</v>
       </c>
       <c r="C89" t="s">
-        <v>59</v>
+        <v>51</v>
       </c>
       <c r="D89" t="s">
         <v>61</v>
       </c>
       <c r="E89">
-        <v>50.4</v>
+        <v>34.729999999999997</v>
       </c>
       <c r="F89">
-        <v>1.94</v>
+        <v>2.87</v>
       </c>
       <c r="G89" t="s">
         <v>53</v>
@@ -9865,7 +10910,7 @@
         <v>2</v>
       </c>
       <c r="J89" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="K89">
         <v>6</v>
@@ -9876,22 +10921,22 @@
     </row>
     <row r="90" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A90" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="B90">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="C90" t="s">
-        <v>59</v>
+        <v>51</v>
       </c>
       <c r="D90" t="s">
         <v>61</v>
       </c>
       <c r="E90">
-        <v>29.06</v>
+        <v>37.799999999999997</v>
       </c>
       <c r="F90">
-        <v>2.0099999999999998</v>
+        <v>2.87</v>
       </c>
       <c r="G90" t="s">
         <v>53</v>
@@ -9903,7 +10948,7 @@
         <v>2</v>
       </c>
       <c r="J90" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="K90">
         <v>6</v>
@@ -9917,19 +10962,19 @@
         <v>10</v>
       </c>
       <c r="B91">
-        <v>2.5</v>
+        <v>3.5</v>
       </c>
       <c r="C91" t="s">
-        <v>59</v>
+        <v>51</v>
       </c>
       <c r="D91" t="s">
         <v>61</v>
       </c>
       <c r="E91">
-        <v>23.67</v>
+        <v>38.75</v>
       </c>
       <c r="F91">
-        <v>1.94</v>
+        <v>2.97</v>
       </c>
       <c r="G91" t="s">
         <v>53</v>
@@ -9941,7 +10986,7 @@
         <v>2</v>
       </c>
       <c r="J91" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="K91">
         <v>6</v>
@@ -9952,22 +10997,22 @@
     </row>
     <row r="92" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A92" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B92">
-        <v>3</v>
+        <v>0.08</v>
       </c>
       <c r="C92" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="D92" t="s">
         <v>61</v>
       </c>
       <c r="E92">
-        <v>31.93</v>
+        <v>16.12</v>
       </c>
       <c r="F92">
-        <v>2.23</v>
+        <v>2.59</v>
       </c>
       <c r="G92" t="s">
         <v>53</v>
@@ -9979,7 +11024,7 @@
         <v>2</v>
       </c>
       <c r="J92" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="K92">
         <v>6</v>
@@ -9990,22 +11035,22 @@
     </row>
     <row r="93" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A93" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B93">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="C93" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="D93" t="s">
         <v>61</v>
       </c>
       <c r="E93">
-        <v>49.39</v>
+        <v>20.14</v>
       </c>
       <c r="F93">
-        <v>1.87</v>
+        <v>2.66</v>
       </c>
       <c r="G93" t="s">
         <v>53</v>
@@ -10017,7 +11062,7 @@
         <v>2</v>
       </c>
       <c r="J93" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="K93">
         <v>6</v>
@@ -10028,22 +11073,22 @@
     </row>
     <row r="94" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A94" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="B94">
         <v>3</v>
       </c>
       <c r="C94" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="D94" t="s">
         <v>61</v>
       </c>
       <c r="E94">
-        <v>32.36</v>
+        <v>25.89</v>
       </c>
       <c r="F94">
-        <v>2.08</v>
+        <v>2.66</v>
       </c>
       <c r="G94" t="s">
         <v>53</v>
@@ -10055,7 +11100,7 @@
         <v>2</v>
       </c>
       <c r="J94" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="K94">
         <v>6</v>
@@ -10069,19 +11114,19 @@
         <v>10</v>
       </c>
       <c r="B95">
-        <v>3</v>
+        <v>3.5</v>
       </c>
       <c r="C95" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="D95" t="s">
         <v>61</v>
       </c>
       <c r="E95">
-        <v>22.8</v>
+        <v>27.76</v>
       </c>
       <c r="F95">
-        <v>2.0099999999999998</v>
+        <v>2.59</v>
       </c>
       <c r="G95" t="s">
         <v>53</v>
@@ -10093,7 +11138,7 @@
         <v>2</v>
       </c>
       <c r="J95" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="K95">
         <v>6</v>
@@ -10104,10 +11149,10 @@
     </row>
     <row r="96" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A96" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B96">
-        <v>3.5</v>
+        <v>0.08</v>
       </c>
       <c r="C96" t="s">
         <v>59</v>
@@ -10116,10 +11161,10 @@
         <v>61</v>
       </c>
       <c r="E96">
-        <v>31.21</v>
+        <v>14.03</v>
       </c>
       <c r="F96">
-        <v>2.37</v>
+        <v>2.0099999999999998</v>
       </c>
       <c r="G96" t="s">
         <v>53</v>
@@ -10142,10 +11187,10 @@
     </row>
     <row r="97" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A97" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B97">
-        <v>3.5</v>
+        <v>2.5</v>
       </c>
       <c r="C97" t="s">
         <v>59</v>
@@ -10154,10 +11199,10 @@
         <v>61</v>
       </c>
       <c r="E97">
-        <v>52.41</v>
+        <v>23.67</v>
       </c>
       <c r="F97">
-        <v>1.87</v>
+        <v>1.94</v>
       </c>
       <c r="G97" t="s">
         <v>53</v>
@@ -10180,10 +11225,10 @@
     </row>
     <row r="98" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A98" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="B98">
-        <v>3.5</v>
+        <v>3</v>
       </c>
       <c r="C98" t="s">
         <v>59</v>
@@ -10192,10 +11237,10 @@
         <v>61</v>
       </c>
       <c r="E98">
-        <v>46.59</v>
+        <v>22.8</v>
       </c>
       <c r="F98">
-        <v>2.08</v>
+        <v>2.0099999999999998</v>
       </c>
       <c r="G98" t="s">
         <v>53</v>
@@ -10255,7 +11300,13 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A3:L3" xr:uid="{DD8C19C1-A04A-491D-9968-DEDC95C2A8FF}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A4:L99">
+      <sortCondition ref="A3"/>
+    </sortState>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>